<commit_message>
prise en compte des retours + refonte id e6ab2a2a3ccbf78e47e1a7a4e62b1d663a89e185
</commit_message>
<xml_diff>
--- a/spec-tech/ig/StructureDefinition-patId.xlsx
+++ b/spec-tech/ig/StructureDefinition-patId.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="99">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-27T13:36:25+00:00</t>
+    <t>2026-07-30T09:32:03+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -81,7 +81,9 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Identifiant du patient tel que connu par les interlocuteurs prenant part à l'échange. Le matricule INS (NIR ou NIA) du patient doit être utilisé en priorité. À défaut de disponibilité de l'INS, un autre identifiant (ex: IPP du système émetteur) peut être utilisé.</t>
+    <t>Identifiant du patient tel que connu par les interlocuteurs prenant part à l'échange. 
+- Matricule INS : le matricule INS (NIR ou NIA) du patient doit être utilisé en priorité. 
+- Autre identifiant : à défaut de disponibilité de l'INS, un autre identifiant (ex: IPP du système émetteur) peut être utilisé.</t>
   </si>
   <si>
     <t>Purpose</t>
@@ -99,16 +101,19 @@
     <t>Kind</t>
   </si>
   <si>
-    <t>logical</t>
+    <t>primitive-type</t>
   </si>
   <si>
     <t>Type</t>
   </si>
   <si>
+    <t>string</t>
+  </si>
+  <si>
     <t>Base Definition</t>
   </si>
   <si>
-    <t>http://hl7.org/fhir/StructureDefinition/Base|4.0.1</t>
+    <t>http://hl7.org/fhir/StructureDefinition/string|4.0.1</t>
   </si>
   <si>
     <t>Abstract</t>
@@ -120,7 +125,7 @@
     <t>Derivation</t>
   </si>
   <si>
-    <t>specialization</t>
+    <t>constraint</t>
   </si>
   <si>
     <t>ID</t>
@@ -229,9 +234,6 @@
   </si>
   <si>
     <t>Constraint(s)</t>
-  </si>
-  <si>
-    <t>patId</t>
   </si>
   <si>
     <t/>
@@ -247,10 +249,20 @@
 </t>
   </si>
   <si>
-    <t>Base</t>
-  </si>
-  <si>
-    <t>patId.patId</t>
+    <t>Primitive Type string</t>
+  </si>
+  <si>
+    <t>A sequence of Unicode characters</t>
+  </si>
+  <si>
+    <t>Note that FHIR strings SHALL NOT exceed 1MB in size</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}
+</t>
+  </si>
+  <si>
+    <t>string.id</t>
   </si>
   <si>
     <t>1</t>
@@ -260,7 +272,52 @@
 </t>
   </si>
   <si>
-    <t>Identifiant du patient. L'INS du patient tel que défini dans le cadre juridique, est à utiliser prioritairement. À défaut, un autre identifiant (ex : IPP du système émetteur) peut être utilisé.</t>
+    <t>xml:id (or equivalent in JSON)</t>
+  </si>
+  <si>
+    <t>unique id for the element within a resource (for internal references)</t>
+  </si>
+  <si>
+    <t>Element.id</t>
+  </si>
+  <si>
+    <t>string.extension</t>
+  </si>
+  <si>
+    <t>extensions
+user content</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extension
+</t>
+  </si>
+  <si>
+    <t>Additional content defined by implementations</t>
+  </si>
+  <si>
+    <t>May be used to represent additional information that is not part of the basic definition of the resource. To make the use of extensions safe and manageable, there is a strict set of governance  applied to the definition and use of extensions. Though any implementer can define an extension, there is a set of requirements that SHALL be met as part of the definition of the extension.</t>
+  </si>
+  <si>
+    <t>There can be no stigma associated with the use of extensions by any application, project, or standard - regardless of the institution or jurisdiction that uses or defines the extensions.  The use of extensions is what allows the FHIR specification to retain a core level of simplicity for everyone.</t>
+  </si>
+  <si>
+    <t>Element.extension</t>
+  </si>
+  <si>
+    <t>ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}
+ext-1:Must have either extensions or value[x], not both {extension.exists() != value.exists()}</t>
+  </si>
+  <si>
+    <t>string.value</t>
+  </si>
+  <si>
+    <t>Primitive value for string</t>
+  </si>
+  <si>
+    <t>The actual value</t>
+  </si>
+  <si>
+    <t>1048576</t>
   </si>
 </sst>
 </file>
@@ -528,31 +585,31 @@
         <v>29</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>3</v>
+        <v>30</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="2">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="2">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -562,20 +619,20 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AJ3"/>
+  <dimension ref="A1:AJ5"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="9.47265625" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="9.47265625" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="13.59765625" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="13.59765625" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="10.8515625" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="4" max="4" width="7.6796875" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="4" max="4" width="10.83984375" customWidth="true" bestFit="true" hidden="true"/>
     <col min="5" max="5" width="5.80859375" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="4.23828125" customWidth="true" bestFit="true"/>
     <col min="7" max="7" width="4.65625" customWidth="true" bestFit="true"/>
     <col min="8" max="8" width="13.953125" customWidth="true" bestFit="true"/>
     <col min="9" max="9" width="11.3671875" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="7.6796875" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="8.609375" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>
@@ -596,7 +653,7 @@
     <col min="29" max="29" width="17.65625" customWidth="true" bestFit="true"/>
     <col min="30" max="30" width="14.7578125" customWidth="true" bestFit="true"/>
     <col min="31" max="31" width="12.359375" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="32" max="32" width="9.91015625" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="32" max="32" width="15.59375" customWidth="true" bestFit="true" hidden="true"/>
     <col min="33" max="33" width="9.046875" customWidth="true" bestFit="true" hidden="true"/>
     <col min="34" max="34" width="9.46484375" customWidth="true" bestFit="true"/>
     <col min="35" max="35" width="100.703125" customWidth="true"/>
@@ -604,120 +661,120 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="1">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B1" t="s" s="1">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C1" t="s" s="1">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D1" t="s" s="1">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E1" t="s" s="1">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F1" t="s" s="1">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G1" t="s" s="1">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H1" t="s" s="1">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="I1" t="s" s="1">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="J1" t="s" s="1">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="K1" t="s" s="1">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="L1" t="s" s="1">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="M1" t="s" s="1">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="N1" t="s" s="1">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="O1" t="s" s="1">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="P1" t="s" s="1">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Q1" t="s" s="1">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="R1" t="s" s="1">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="S1" t="s" s="1">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="T1" t="s" s="1">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="U1" t="s" s="1">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="V1" t="s" s="1">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="W1" t="s" s="1">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="X1" t="s" s="1">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="Y1" t="s" s="1">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="Z1" t="s" s="1">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="AA1" t="s" s="1">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="AB1" t="s" s="1">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="AC1" t="s" s="1">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AD1" t="s" s="1">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="AE1" t="s" s="1">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="AF1" t="s" s="1">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="AG1" t="s" s="1">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="AH1" t="s" s="1">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="AI1" t="s" s="1">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="AJ1" t="s" s="1">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="2">
-        <v>72</v>
+        <v>30</v>
       </c>
       <c r="B2" t="s" s="2">
-        <v>72</v>
+        <v>30</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" t="s" s="2">
@@ -743,12 +800,14 @@
         <v>76</v>
       </c>
       <c r="L2" t="s" s="2">
-        <v>9</v>
+        <v>77</v>
       </c>
       <c r="M2" t="s" s="2">
-        <v>22</v>
-      </c>
-      <c r="N2" s="2"/>
+        <v>78</v>
+      </c>
+      <c r="N2" t="s" s="2">
+        <v>79</v>
+      </c>
       <c r="O2" s="2"/>
       <c r="P2" t="s" s="2">
         <v>73</v>
@@ -797,7 +856,7 @@
         <v>73</v>
       </c>
       <c r="AF2" t="s" s="2">
-        <v>77</v>
+        <v>30</v>
       </c>
       <c r="AG2" t="s" s="2">
         <v>74</v>
@@ -809,15 +868,15 @@
         <v>73</v>
       </c>
       <c r="AJ2" t="s" s="2">
-        <v>73</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="2">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B3" t="s" s="2">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" t="s" s="2">
@@ -825,10 +884,10 @@
       </c>
       <c r="E3" s="2"/>
       <c r="F3" t="s" s="2">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="G3" t="s" s="2">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="H3" t="s" s="2">
         <v>73</v>
@@ -840,13 +899,13 @@
         <v>73</v>
       </c>
       <c r="K3" t="s" s="2">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="L3" t="s" s="2">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="M3" t="s" s="2">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="N3" s="2"/>
       <c r="O3" s="2"/>
@@ -897,18 +956,220 @@
         <v>73</v>
       </c>
       <c r="AF3" t="s" s="2">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="AG3" t="s" s="2">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="AH3" t="s" s="2">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="AI3" t="s" s="2">
         <v>73</v>
       </c>
       <c r="AJ3" t="s" s="2">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="B4" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="C4" s="2"/>
+      <c r="D4" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="E4" s="2"/>
+      <c r="F4" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="G4" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="H4" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="I4" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="J4" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="K4" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="L4" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="M4" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="N4" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="O4" s="2"/>
+      <c r="P4" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Q4" s="2"/>
+      <c r="R4" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="S4" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="T4" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="U4" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="V4" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="W4" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="X4" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Y4" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Z4" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AA4" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AB4" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AC4" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AD4" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AE4" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AF4" t="s" s="2">
+        <v>93</v>
+      </c>
+      <c r="AG4" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AH4" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AI4" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AJ4" t="s" s="2">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="2">
+        <v>95</v>
+      </c>
+      <c r="B5" t="s" s="2">
+        <v>95</v>
+      </c>
+      <c r="C5" s="2"/>
+      <c r="D5" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="E5" s="2"/>
+      <c r="F5" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="G5" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="H5" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="I5" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="J5" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="K5" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="L5" t="s" s="2">
+        <v>96</v>
+      </c>
+      <c r="M5" t="s" s="2">
+        <v>97</v>
+      </c>
+      <c r="N5" s="2"/>
+      <c r="O5" s="2"/>
+      <c r="P5" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Q5" s="2"/>
+      <c r="R5" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="S5" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="T5" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="U5" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="V5" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="W5" t="s" s="2">
+        <v>98</v>
+      </c>
+      <c r="X5" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Y5" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Z5" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AA5" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AB5" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AC5" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AD5" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AE5" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AF5" t="s" s="2">
+        <v>95</v>
+      </c>
+      <c r="AG5" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AH5" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AI5" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AJ5" t="s" s="2">
         <v>73</v>
       </c>
     </row>

</xml_diff>